<commit_message>
Redesign: temporal slider, IDS ranking, new UI, updated indicators
</commit_message>
<xml_diff>
--- a/data/indicadores/01_04_02_05_ssb.xlsx
+++ b/data/indicadores/01_04_02_05_ssb.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\INDICADORES Y DEMAS 2026 EN ESCRITORIO\3 INDICADORS SB\2012 y 2024 LYKE\URB RUR INE\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\INDICADORES Y DEMAS 2026 EN ESCRITORIO\OFICIALES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A005836-E1FF-423B-8626-1DEFBB6CC3CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCAC97C0-DC6F-4364-A2B7-399F9675D778}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="802" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5947,41 +5947,42 @@
         <v>10101</v>
       </c>
       <c r="F4" s="2">
-        <v>3414</v>
+        <v>3453</v>
       </c>
       <c r="G4" s="2">
-        <v>4020</v>
+        <v>4030</v>
       </c>
       <c r="H4" s="2">
-        <v>8057</v>
+        <v>8093</v>
       </c>
       <c r="I4" s="2">
-        <v>54344</v>
+        <v>54373</v>
       </c>
       <c r="J4" s="2">
-        <v>69835</v>
+        <v>69949</v>
       </c>
       <c r="K4" s="3">
         <f>(I4/J4)*100</f>
-        <v>77.817713181069664</v>
+        <v>77.732347853436082</v>
       </c>
       <c r="L4" s="2">
-        <v>3414</v>
-      </c>
+        <v>3453</v>
+      </c>
+      <c r="M4" s="38"/>
       <c r="P4" s="25" t="s">
         <v>20</v>
       </c>
       <c r="Q4" s="43">
         <f>+SUM(F4:F32)</f>
-        <v>26012</v>
+        <v>25961</v>
       </c>
       <c r="R4" s="43">
         <f t="shared" ref="R4:U4" si="0">+SUM(G4:G32)</f>
-        <v>24095</v>
+        <v>24030</v>
       </c>
       <c r="S4" s="43">
         <f t="shared" si="0"/>
-        <v>24808</v>
+        <v>24803</v>
       </c>
       <c r="T4" s="43">
         <f t="shared" si="0"/>
@@ -5989,15 +5990,15 @@
       </c>
       <c r="U4" s="43">
         <f t="shared" si="0"/>
-        <v>150202</v>
+        <v>150081</v>
       </c>
       <c r="V4" s="45">
         <f t="shared" ref="V4:V12" si="1">(T4/U4)*100</f>
-        <v>50.12383323790629</v>
+        <v>50.164244641227071</v>
       </c>
       <c r="W4" s="43">
-        <f t="shared" ref="W4:W12" si="2">U4-T4</f>
-        <v>74915</v>
+        <f>U4-T4</f>
+        <v>74794</v>
       </c>
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.25">
@@ -6032,7 +6033,7 @@
         <v>2646</v>
       </c>
       <c r="K5" s="3">
-        <f t="shared" ref="K5:K68" si="3">(I5/J5)*100</f>
+        <f t="shared" ref="K5:K68" si="2">(I5/J5)*100</f>
         <v>44.897959183673471</v>
       </c>
       <c r="L5" s="2">
@@ -6046,19 +6047,19 @@
         <v>79253</v>
       </c>
       <c r="R5" s="44">
-        <f t="shared" ref="R5:U5" si="4">+SUM(G33:G119)</f>
+        <f t="shared" ref="R5:U5" si="3">+SUM(G33:G119)</f>
         <v>118358</v>
       </c>
       <c r="S5" s="44">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>205296</v>
       </c>
       <c r="T5" s="44">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>449666</v>
       </c>
       <c r="U5" s="44">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>852573</v>
       </c>
       <c r="V5" s="45">
@@ -6066,7 +6067,7 @@
         <v>52.742228524712843</v>
       </c>
       <c r="W5" s="43">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="W5:W12" si="4">U5-T5</f>
         <v>402907</v>
       </c>
     </row>
@@ -6087,57 +6088,57 @@
         <v>10103</v>
       </c>
       <c r="F6" s="2">
-        <v>2634</v>
+        <v>2544</v>
       </c>
       <c r="G6" s="2">
-        <v>1660</v>
+        <v>1585</v>
       </c>
       <c r="H6" s="2">
-        <v>396</v>
+        <v>355</v>
       </c>
       <c r="I6" s="2">
-        <v>205</v>
+        <v>176</v>
       </c>
       <c r="J6" s="2">
-        <v>4895</v>
+        <v>4660</v>
       </c>
       <c r="K6" s="3">
-        <f t="shared" si="3"/>
-        <v>4.1879468845760979</v>
+        <f t="shared" si="2"/>
+        <v>3.7768240343347639</v>
       </c>
       <c r="L6" s="2">
-        <v>2634</v>
+        <v>2544</v>
       </c>
       <c r="P6" s="25" t="s">
         <v>3</v>
       </c>
       <c r="Q6" s="44">
         <f>+SUM(F120:F167)</f>
-        <v>59642</v>
+        <v>57060</v>
       </c>
       <c r="R6" s="44">
         <f t="shared" ref="R6:U6" si="5">+SUM(G120:G167)</f>
-        <v>110687</v>
+        <v>108872</v>
       </c>
       <c r="S6" s="44">
         <f t="shared" si="5"/>
-        <v>135003</v>
+        <v>132705</v>
       </c>
       <c r="T6" s="44">
         <f t="shared" si="5"/>
-        <v>219187</v>
+        <v>217971</v>
       </c>
       <c r="U6" s="44">
         <f t="shared" si="5"/>
-        <v>524519</v>
+        <v>516608</v>
       </c>
       <c r="V6" s="45">
         <f t="shared" si="1"/>
-        <v>41.788190704245224</v>
+        <v>42.192726399900891</v>
       </c>
       <c r="W6" s="43">
-        <f t="shared" si="2"/>
-        <v>305332</v>
+        <f t="shared" si="4"/>
+        <v>298637</v>
       </c>
     </row>
     <row r="7" spans="1:23" x14ac:dyDescent="0.25">
@@ -6172,7 +6173,7 @@
         <v>2538</v>
       </c>
       <c r="K7" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>12.844759653270291</v>
       </c>
       <c r="L7" s="2">
@@ -6206,7 +6207,7 @@
         <v>41.639868210783831</v>
       </c>
       <c r="W7" s="43">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>88743</v>
       </c>
     </row>
@@ -6242,7 +6243,7 @@
         <v>3418</v>
       </c>
       <c r="K8" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>13.136337039204212</v>
       </c>
       <c r="L8" s="2">
@@ -6253,31 +6254,31 @@
       </c>
       <c r="Q8" s="44">
         <f>+SUM(F203:F244)</f>
-        <v>39275</v>
+        <v>35584</v>
       </c>
       <c r="R8" s="44">
         <f t="shared" ref="R8:U8" si="7">+SUM(G203:G244)</f>
-        <v>56795</v>
+        <v>51949</v>
       </c>
       <c r="S8" s="44">
         <f t="shared" si="7"/>
-        <v>72076</v>
+        <v>66660</v>
       </c>
       <c r="T8" s="44">
         <f t="shared" si="7"/>
-        <v>89901</v>
+        <v>88109</v>
       </c>
       <c r="U8" s="44">
         <f t="shared" si="7"/>
-        <v>258047</v>
+        <v>242302</v>
       </c>
       <c r="V8" s="45">
         <f t="shared" si="1"/>
-        <v>34.839002197274141</v>
+        <v>36.363298693366133</v>
       </c>
       <c r="W8" s="43">
-        <f t="shared" si="2"/>
-        <v>168146</v>
+        <f t="shared" si="4"/>
+        <v>154193</v>
       </c>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.25">
@@ -6312,7 +6313,7 @@
         <v>2586</v>
       </c>
       <c r="K9" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>27.803557617942769</v>
       </c>
       <c r="L9" s="2">
@@ -6346,7 +6347,7 @@
         <v>67.17492554337494</v>
       </c>
       <c r="W9" s="43">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>41441</v>
       </c>
     </row>
@@ -6382,7 +6383,7 @@
         <v>2717</v>
       </c>
       <c r="K10" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>17.372101582627899</v>
       </c>
       <c r="L10" s="2">
@@ -6416,7 +6417,7 @@
         <v>43.773009084226814</v>
       </c>
       <c r="W10" s="43">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>362582</v>
       </c>
     </row>
@@ -6452,7 +6453,7 @@
         <v>1982</v>
       </c>
       <c r="K11" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>26.892028254288597</v>
       </c>
       <c r="L11" s="2">
@@ -6463,31 +6464,31 @@
       </c>
       <c r="Q11" s="44">
         <f>+SUM(F312:F331)</f>
-        <v>8068</v>
+        <v>7636</v>
       </c>
       <c r="R11" s="44">
         <f t="shared" ref="R11:U11" si="10">+SUM(G312:G331)</f>
-        <v>32496</v>
+        <v>31214</v>
       </c>
       <c r="S11" s="44">
         <f t="shared" si="10"/>
-        <v>36967.5</v>
+        <v>35542</v>
       </c>
       <c r="T11" s="44">
         <f t="shared" si="10"/>
-        <v>20391.5</v>
+        <v>19498</v>
       </c>
       <c r="U11" s="44">
         <f t="shared" si="10"/>
-        <v>97923</v>
+        <v>93890</v>
       </c>
       <c r="V11" s="45">
         <f t="shared" si="1"/>
-        <v>20.824014787128661</v>
+        <v>20.766854830120355</v>
       </c>
       <c r="W11" s="43">
-        <f t="shared" si="2"/>
-        <v>77531.5</v>
+        <f t="shared" si="4"/>
+        <v>74392</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
@@ -6522,7 +6523,7 @@
         <v>1831</v>
       </c>
       <c r="K12" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>39.377389404696892</v>
       </c>
       <c r="L12" s="2">
@@ -6556,7 +6557,7 @@
         <v>19.246993889217425</v>
       </c>
       <c r="W12" s="59">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>20483</v>
       </c>
     </row>
@@ -6592,7 +6593,7 @@
         <v>2810</v>
       </c>
       <c r="K13" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>33.45195729537366</v>
       </c>
       <c r="L13" s="2">
@@ -6620,7 +6621,7 @@
         <v>65.076052935039257</v>
       </c>
       <c r="W13" s="21">
-        <v>12720</v>
+        <v>801</v>
       </c>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.25">
@@ -6655,7 +6656,7 @@
         <v>2113</v>
       </c>
       <c r="K14" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>28.064363464268808</v>
       </c>
       <c r="L14" s="2">
@@ -6666,31 +6667,31 @@
       </c>
       <c r="Q14" s="21">
         <f>SUM(Q4:Q12)</f>
-        <v>258487</v>
+        <v>251731</v>
       </c>
       <c r="R14" s="21">
-        <f t="shared" ref="R14:W14" si="12">SUM(R4:R12)</f>
-        <v>422565</v>
+        <f t="shared" ref="R14:U14" si="12">SUM(R4:R12)</f>
+        <v>414557</v>
       </c>
       <c r="S14" s="21">
         <f t="shared" si="12"/>
-        <v>861028.5</v>
+        <v>851884</v>
       </c>
       <c r="T14" s="21">
         <f t="shared" si="12"/>
-        <v>1289711.5</v>
+        <v>1285810</v>
       </c>
       <c r="U14" s="21">
         <f t="shared" si="12"/>
-        <v>2831792</v>
+        <v>2803982</v>
       </c>
       <c r="V14" s="61">
         <f>(T14/U14)*100</f>
-        <v>45.544005350675477</v>
+        <v>45.856571119215459</v>
       </c>
       <c r="W14" s="21">
-        <f t="shared" si="12"/>
-        <v>1542080.5</v>
+        <f>SUM(W4:W12)</f>
+        <v>1518172</v>
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
@@ -6725,7 +6726,7 @@
         <v>2010</v>
       </c>
       <c r="K15" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>26.766169154228859</v>
       </c>
       <c r="L15" s="2">
@@ -6764,7 +6765,7 @@
         <v>1072</v>
       </c>
       <c r="K16" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>22.761194029850746</v>
       </c>
       <c r="L16" s="2">
@@ -6803,7 +6804,7 @@
         <v>1212</v>
       </c>
       <c r="K17" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>22.112211221122113</v>
       </c>
       <c r="L17" s="2">
@@ -6842,7 +6843,7 @@
         <v>6079</v>
       </c>
       <c r="K18" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>46.718210231946045</v>
       </c>
       <c r="L18" s="2">
@@ -6881,7 +6882,7 @@
         <v>2079</v>
       </c>
       <c r="K19" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>26.936026936026934</v>
       </c>
       <c r="L19" s="2">
@@ -6920,7 +6921,7 @@
         <v>4386</v>
       </c>
       <c r="K20" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>19.33424532603739</v>
       </c>
       <c r="L20" s="2">
@@ -6959,7 +6960,7 @@
         <v>2950</v>
       </c>
       <c r="K21" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>20.711864406779661</v>
       </c>
       <c r="L21" s="2">
@@ -6998,7 +6999,7 @@
         <v>4325</v>
       </c>
       <c r="K22" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>42.01156069364162</v>
       </c>
       <c r="L22" s="2">
@@ -7037,7 +7038,7 @@
         <v>8008</v>
       </c>
       <c r="K23" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>16.058941058941059</v>
       </c>
       <c r="L23" s="2">
@@ -7076,7 +7077,7 @@
         <v>2779</v>
       </c>
       <c r="K24" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>13.781935948182799</v>
       </c>
       <c r="L24" s="2">
@@ -7115,7 +7116,7 @@
         <v>3475</v>
       </c>
       <c r="K25" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>15.827338129496402</v>
       </c>
       <c r="L25" s="2">
@@ -7154,7 +7155,7 @@
         <v>3196</v>
       </c>
       <c r="K26" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>40.425531914893611</v>
       </c>
       <c r="L26" s="2">
@@ -7193,7 +7194,7 @@
         <v>965</v>
       </c>
       <c r="K27" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>26.735751295336783</v>
       </c>
       <c r="L27" s="2">
@@ -7232,7 +7233,7 @@
         <v>4347</v>
       </c>
       <c r="K28" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>26.455026455026452</v>
       </c>
       <c r="L28" s="2">
@@ -7271,7 +7272,7 @@
         <v>1062</v>
       </c>
       <c r="K29" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>35.969868173258</v>
       </c>
       <c r="L29" s="2">
@@ -7310,7 +7311,7 @@
         <v>2532</v>
       </c>
       <c r="K30" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>39.889415481832543</v>
       </c>
       <c r="L30" s="2">
@@ -7349,7 +7350,7 @@
         <v>603</v>
       </c>
       <c r="K31" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>23.217247097844112</v>
       </c>
       <c r="L31" s="2">
@@ -7388,7 +7389,7 @@
         <v>1751</v>
       </c>
       <c r="K32" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>35.408338092518562</v>
       </c>
       <c r="L32" s="2">
@@ -7427,7 +7428,7 @@
         <v>226458</v>
       </c>
       <c r="K33" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>89.065522083565156</v>
       </c>
       <c r="L33" s="2">
@@ -7466,7 +7467,7 @@
         <v>4853</v>
       </c>
       <c r="K34" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>15.516175561508344</v>
       </c>
       <c r="L34" s="2">
@@ -7490,26 +7491,26 @@
         <v>20103</v>
       </c>
       <c r="F35" s="2">
-        <v>508</v>
+        <v>504</v>
       </c>
       <c r="G35" s="2">
-        <v>1474</v>
+        <v>1466</v>
       </c>
       <c r="H35" s="2">
-        <v>1307</v>
+        <v>1254</v>
       </c>
       <c r="I35" s="2">
-        <v>1549</v>
+        <v>1548</v>
       </c>
       <c r="J35" s="2">
-        <v>4838</v>
+        <v>4772</v>
       </c>
       <c r="K35" s="3">
-        <f t="shared" si="3"/>
-        <v>32.017362546506824</v>
+        <f t="shared" si="2"/>
+        <v>32.439228834870079</v>
       </c>
       <c r="L35" s="2">
-        <v>508</v>
+        <v>504</v>
       </c>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.25">
@@ -7529,26 +7530,26 @@
         <v>20104</v>
       </c>
       <c r="F36" s="2">
-        <v>1231</v>
+        <v>1235</v>
       </c>
       <c r="G36" s="2">
-        <v>3113</v>
+        <v>3121</v>
       </c>
       <c r="H36" s="2">
-        <v>2261</v>
+        <v>2314</v>
       </c>
       <c r="I36" s="2">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="J36" s="2">
-        <v>7085</v>
+        <v>7151</v>
       </c>
       <c r="K36" s="3">
-        <f t="shared" si="3"/>
-        <v>6.7748764996471422</v>
+        <f t="shared" si="2"/>
+        <v>6.7263319815410432</v>
       </c>
       <c r="L36" s="2">
-        <v>1231</v>
+        <v>1235</v>
       </c>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.25">
@@ -7583,7 +7584,7 @@
         <v>256852</v>
       </c>
       <c r="K37" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>63.026957158207843</v>
       </c>
       <c r="L37" s="2">
@@ -7622,7 +7623,7 @@
         <v>16228</v>
       </c>
       <c r="K38" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>38.180921863445896</v>
       </c>
       <c r="L38" s="2">
@@ -7661,7 +7662,7 @@
         <v>5027</v>
       </c>
       <c r="K39" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>14.442013129102845</v>
       </c>
       <c r="L39" s="2">
@@ -7685,26 +7686,26 @@
         <v>20203</v>
       </c>
       <c r="F40" s="2">
-        <v>83</v>
+        <v>547</v>
       </c>
       <c r="G40" s="2">
-        <v>237</v>
+        <v>914</v>
       </c>
       <c r="H40" s="2">
-        <v>479</v>
+        <v>1091</v>
       </c>
       <c r="I40" s="2">
-        <v>863</v>
+        <v>745</v>
       </c>
       <c r="J40" s="2">
-        <v>1662</v>
+        <v>3297</v>
       </c>
       <c r="K40" s="3">
-        <f t="shared" si="3"/>
-        <v>51.925391095066189</v>
+        <f t="shared" si="2"/>
+        <v>22.596299666363361</v>
       </c>
       <c r="L40" s="2">
-        <v>83</v>
+        <v>547</v>
       </c>
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.25">
@@ -7724,26 +7725,26 @@
         <v>20204</v>
       </c>
       <c r="F41" s="2">
-        <v>193</v>
+        <v>485</v>
       </c>
       <c r="G41" s="2">
-        <v>398</v>
+        <v>764</v>
       </c>
       <c r="H41" s="2">
-        <v>842</v>
+        <v>1229</v>
       </c>
       <c r="I41" s="2">
-        <v>599</v>
+        <v>1319</v>
       </c>
       <c r="J41" s="2">
-        <v>2032</v>
+        <v>3797</v>
       </c>
       <c r="K41" s="3">
-        <f t="shared" si="3"/>
-        <v>29.478346456692911</v>
+        <f t="shared" si="2"/>
+        <v>34.737951013958387</v>
       </c>
       <c r="L41" s="2">
-        <v>193</v>
+        <v>485</v>
       </c>
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.25">
@@ -7763,26 +7764,26 @@
         <v>20205</v>
       </c>
       <c r="F42" s="2">
-        <v>547</v>
+        <v>83</v>
       </c>
       <c r="G42" s="2">
-        <v>914</v>
+        <v>237</v>
       </c>
       <c r="H42" s="2">
-        <v>1091</v>
+        <v>479</v>
       </c>
       <c r="I42" s="2">
-        <v>745</v>
+        <v>863</v>
       </c>
       <c r="J42" s="2">
-        <v>3297</v>
+        <v>1662</v>
       </c>
       <c r="K42" s="3">
-        <f t="shared" si="3"/>
-        <v>22.596299666363361</v>
+        <f t="shared" si="2"/>
+        <v>51.925391095066189</v>
       </c>
       <c r="L42" s="2">
-        <v>547</v>
+        <v>83</v>
       </c>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.25">
@@ -7802,26 +7803,26 @@
         <v>20206</v>
       </c>
       <c r="F43" s="2">
-        <v>485</v>
+        <v>193</v>
       </c>
       <c r="G43" s="2">
-        <v>764</v>
+        <v>398</v>
       </c>
       <c r="H43" s="2">
-        <v>1229</v>
+        <v>842</v>
       </c>
       <c r="I43" s="2">
-        <v>1319</v>
+        <v>599</v>
       </c>
       <c r="J43" s="2">
-        <v>3797</v>
+        <v>2032</v>
       </c>
       <c r="K43" s="3">
-        <f t="shared" si="3"/>
-        <v>34.737951013958387</v>
+        <f t="shared" si="2"/>
+        <v>29.478346456692911</v>
       </c>
       <c r="L43" s="2">
-        <v>485</v>
+        <v>193</v>
       </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.25">
@@ -7856,7 +7857,7 @@
         <v>3740</v>
       </c>
       <c r="K44" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>9.3850267379679142</v>
       </c>
       <c r="L44" s="2">
@@ -7895,7 +7896,7 @@
         <v>4269</v>
       </c>
       <c r="K45" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>10.260014054813773</v>
       </c>
       <c r="L45" s="2">
@@ -7934,7 +7935,7 @@
         <v>3533</v>
       </c>
       <c r="K46" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>6.057175205208039</v>
       </c>
       <c r="L46" s="2">
@@ -7973,7 +7974,7 @@
         <v>1311</v>
       </c>
       <c r="K47" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>10.526315789473683</v>
       </c>
       <c r="L47" s="2">
@@ -8012,7 +8013,7 @@
         <v>1159</v>
       </c>
       <c r="K48" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>9.9223468507333905</v>
       </c>
       <c r="L48" s="2">
@@ -8051,7 +8052,7 @@
         <v>1070</v>
       </c>
       <c r="K49" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>3.4579439252336446</v>
       </c>
       <c r="L49" s="2">
@@ -8090,7 +8091,7 @@
         <v>289</v>
       </c>
       <c r="K50" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>17.647058823529413</v>
       </c>
       <c r="L50" s="2">
@@ -8129,7 +8130,7 @@
         <v>2790</v>
       </c>
       <c r="K51" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>1.0035842293906809</v>
       </c>
       <c r="L51" s="2">
@@ -8168,7 +8169,7 @@
         <v>5011</v>
       </c>
       <c r="K52" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>10.995809219716623</v>
       </c>
       <c r="L52" s="2">
@@ -8207,7 +8208,7 @@
         <v>6606</v>
       </c>
       <c r="K53" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>16.969421737814109</v>
       </c>
       <c r="L53" s="2">
@@ -8246,7 +8247,7 @@
         <v>5347</v>
       </c>
       <c r="K54" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>15.934168692724892</v>
       </c>
       <c r="L54" s="2">
@@ -8285,7 +8286,7 @@
         <v>2108</v>
       </c>
       <c r="K55" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>13.42504743833017</v>
       </c>
       <c r="L55" s="2">
@@ -8324,7 +8325,7 @@
         <v>3027</v>
       </c>
       <c r="K56" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>9.7125867195242819</v>
       </c>
       <c r="L56" s="2">
@@ -8363,7 +8364,7 @@
         <v>3938</v>
       </c>
       <c r="K57" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>23.743016759776538</v>
       </c>
       <c r="L57" s="2">
@@ -8402,7 +8403,7 @@
         <v>2747</v>
       </c>
       <c r="K58" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>24.899890789952675</v>
       </c>
       <c r="L58" s="2">
@@ -8441,7 +8442,7 @@
         <v>1938</v>
       </c>
       <c r="K59" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>17.595459236326107</v>
       </c>
       <c r="L59" s="2">
@@ -8480,7 +8481,7 @@
         <v>8775</v>
       </c>
       <c r="K60" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>26.210826210826209</v>
       </c>
       <c r="L60" s="2">
@@ -8519,7 +8520,7 @@
         <v>4681</v>
       </c>
       <c r="K61" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>32.236701559495835</v>
       </c>
       <c r="L61" s="2">
@@ -8558,7 +8559,7 @@
         <v>2980</v>
       </c>
       <c r="K62" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>21.107382550335572</v>
       </c>
       <c r="L62" s="2">
@@ -8597,7 +8598,7 @@
         <v>1027</v>
       </c>
       <c r="K63" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>19.766309639727361</v>
       </c>
       <c r="L63" s="2">
@@ -8636,7 +8637,7 @@
         <v>994</v>
       </c>
       <c r="K64" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>23.74245472837022</v>
       </c>
       <c r="L64" s="2">
@@ -8675,7 +8676,7 @@
         <v>3457</v>
       </c>
       <c r="K65" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>26.149840902516637</v>
       </c>
       <c r="L65" s="2">
@@ -8714,7 +8715,7 @@
         <v>4050</v>
       </c>
       <c r="K66" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>21.283950617283949</v>
       </c>
       <c r="L66" s="2">
@@ -8753,7 +8754,7 @@
         <v>3487</v>
       </c>
       <c r="K67" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>23.343848580441641</v>
       </c>
       <c r="L67" s="2">
@@ -8792,7 +8793,7 @@
         <v>4625</v>
       </c>
       <c r="K68" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>26.356756756756756</v>
       </c>
       <c r="L68" s="2">
@@ -9752,26 +9753,26 @@
         <v>21201</v>
       </c>
       <c r="F93" s="2">
-        <v>2291</v>
+        <v>2422</v>
       </c>
       <c r="G93" s="2">
-        <v>2682</v>
+        <v>2950</v>
       </c>
       <c r="H93" s="2">
-        <v>3621</v>
+        <v>3759</v>
       </c>
       <c r="I93" s="2">
-        <v>1967</v>
+        <v>1990</v>
       </c>
       <c r="J93" s="2">
-        <v>10561</v>
+        <v>11121</v>
       </c>
       <c r="K93" s="3">
         <f t="shared" si="13"/>
-        <v>18.625130196004168</v>
+        <v>17.894074273896234</v>
       </c>
       <c r="L93" s="2">
-        <v>2291</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="94" spans="1:12" x14ac:dyDescent="0.25">
@@ -9869,26 +9870,26 @@
         <v>21204</v>
       </c>
       <c r="F96" s="2">
-        <v>341</v>
+        <v>210</v>
       </c>
       <c r="G96" s="2">
-        <v>893</v>
+        <v>625</v>
       </c>
       <c r="H96" s="2">
-        <v>1307</v>
+        <v>1169</v>
       </c>
       <c r="I96" s="2">
-        <v>367</v>
+        <v>344</v>
       </c>
       <c r="J96" s="2">
-        <v>2908</v>
+        <v>2348</v>
       </c>
       <c r="K96" s="3">
         <f t="shared" si="13"/>
-        <v>12.620357634112791</v>
+        <v>14.650766609880749</v>
       </c>
       <c r="L96" s="2">
-        <v>341</v>
+        <v>210</v>
       </c>
     </row>
     <row r="97" spans="1:12" x14ac:dyDescent="0.25">
@@ -12209,26 +12210,26 @@
         <v>31301</v>
       </c>
       <c r="F156" s="2">
-        <v>2582</v>
+        <v>1333</v>
       </c>
       <c r="G156" s="2">
-        <v>1815</v>
+        <v>1311</v>
       </c>
       <c r="H156" s="2">
-        <v>2298</v>
+        <v>2084</v>
       </c>
       <c r="I156" s="2">
-        <v>1216</v>
+        <v>1192</v>
       </c>
       <c r="J156" s="2">
-        <v>7911</v>
+        <v>5920</v>
       </c>
       <c r="K156" s="3">
         <f t="shared" si="14"/>
-        <v>15.371002401719124</v>
+        <v>20.135135135135133</v>
       </c>
       <c r="L156" s="2">
-        <v>2582</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="157" spans="1:12" x14ac:dyDescent="0.25">
@@ -12326,26 +12327,26 @@
         <v>31304</v>
       </c>
       <c r="F159" s="2">
-        <v>2582</v>
+        <v>1249</v>
       </c>
       <c r="G159" s="2">
-        <v>1815</v>
+        <v>504</v>
       </c>
       <c r="H159" s="2">
-        <v>2298</v>
+        <v>214</v>
       </c>
       <c r="I159" s="2">
-        <v>1216</v>
+        <v>24</v>
       </c>
       <c r="J159" s="2">
-        <v>7911</v>
+        <v>1991</v>
       </c>
       <c r="K159" s="3">
         <f t="shared" ref="K159" si="15">(I159/J159)*100</f>
-        <v>15.371002401719124</v>
+        <v>1.2054244098442994</v>
       </c>
       <c r="L159" s="2">
-        <v>2582</v>
+        <v>1249</v>
       </c>
     </row>
     <row r="160" spans="1:12" x14ac:dyDescent="0.25">
@@ -12833,26 +12834,26 @@
         <v>40201</v>
       </c>
       <c r="F172" s="2">
-        <v>1808</v>
+        <v>1815</v>
       </c>
       <c r="G172" s="2">
-        <v>2282</v>
+        <v>2328</v>
       </c>
       <c r="H172" s="2">
-        <v>3274</v>
+        <v>3403</v>
       </c>
       <c r="I172" s="2">
-        <v>2305</v>
+        <v>2327</v>
       </c>
       <c r="J172" s="2">
-        <v>9669</v>
+        <v>9873</v>
       </c>
       <c r="K172" s="3">
         <f t="shared" si="14"/>
-        <v>23.839073327127934</v>
+        <v>23.569330497315914</v>
       </c>
       <c r="L172" s="2">
-        <v>1808</v>
+        <v>1815</v>
       </c>
     </row>
     <row r="173" spans="1:12" x14ac:dyDescent="0.25">
@@ -13847,26 +13848,26 @@
         <v>41401</v>
       </c>
       <c r="F198" s="2">
-        <v>1140</v>
+        <v>1133</v>
       </c>
       <c r="G198" s="2">
-        <v>1127</v>
+        <v>1081</v>
       </c>
       <c r="H198" s="2">
-        <v>1384</v>
+        <v>1255</v>
       </c>
       <c r="I198" s="2">
-        <v>855</v>
+        <v>833</v>
       </c>
       <c r="J198" s="2">
-        <v>4506</v>
+        <v>4302</v>
       </c>
       <c r="K198" s="3">
         <f t="shared" ref="K198:K263" si="16">(I198/J198)*100</f>
-        <v>18.974700399467377</v>
+        <v>19.363086936308694</v>
       </c>
       <c r="L198" s="2">
-        <v>1140</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="199" spans="1:12" x14ac:dyDescent="0.25">
@@ -14471,26 +14472,26 @@
         <v>50401</v>
       </c>
       <c r="F214" s="2">
-        <v>2161</v>
+        <v>919</v>
       </c>
       <c r="G214" s="2">
-        <v>3536</v>
+        <v>1384</v>
       </c>
       <c r="H214" s="2">
-        <v>3460</v>
+        <v>1308</v>
       </c>
       <c r="I214" s="2">
-        <v>1493</v>
+        <v>675</v>
       </c>
       <c r="J214" s="2">
-        <v>10650</v>
+        <v>4286</v>
       </c>
       <c r="K214" s="3">
         <f t="shared" si="16"/>
-        <v>14.018779342723004</v>
+        <v>15.748950069995335</v>
       </c>
       <c r="L214" s="2">
-        <v>2161</v>
+        <v>919</v>
       </c>
     </row>
     <row r="215" spans="1:12" x14ac:dyDescent="0.25">
@@ -14510,26 +14511,26 @@
         <v>50402</v>
       </c>
       <c r="F215" s="2">
-        <v>1613</v>
+        <v>1664</v>
       </c>
       <c r="G215" s="2">
-        <v>2397</v>
+        <v>2462</v>
       </c>
       <c r="H215" s="2">
-        <v>1508</v>
+        <v>1513</v>
       </c>
       <c r="I215" s="2">
         <v>1046</v>
       </c>
       <c r="J215" s="2">
-        <v>6564</v>
+        <v>6685</v>
       </c>
       <c r="K215" s="3">
         <f t="shared" si="16"/>
-        <v>15.935405240706885</v>
+        <v>15.646970830216903</v>
       </c>
       <c r="L215" s="2">
-        <v>1613</v>
+        <v>1664</v>
       </c>
     </row>
     <row r="216" spans="1:12" x14ac:dyDescent="0.25">
@@ -14627,25 +14628,25 @@
         <v>50405</v>
       </c>
       <c r="F218" s="2">
-        <v>2161</v>
+        <v>1242</v>
       </c>
       <c r="G218" s="2">
-        <v>3536</v>
+        <v>2152</v>
       </c>
       <c r="H218" s="2">
-        <v>3460</v>
+        <v>2152</v>
       </c>
       <c r="I218" s="2">
-        <v>1493</v>
+        <v>818</v>
       </c>
       <c r="J218" s="2">
-        <v>10650</v>
+        <v>6364</v>
       </c>
       <c r="K218" s="3">
         <v>14.018779342723004</v>
       </c>
       <c r="L218" s="2">
-        <v>2161</v>
+        <v>1242</v>
       </c>
     </row>
     <row r="219" spans="1:12" x14ac:dyDescent="0.25">
@@ -15328,26 +15329,26 @@
         <v>51202</v>
       </c>
       <c r="F236" s="2">
-        <v>1581</v>
+        <v>951</v>
       </c>
       <c r="G236" s="2">
-        <v>1375</v>
+        <v>849</v>
       </c>
       <c r="H236" s="2">
-        <v>1961</v>
+        <v>1119</v>
       </c>
       <c r="I236" s="2">
-        <v>299</v>
+        <v>158</v>
       </c>
       <c r="J236" s="2">
-        <v>5216</v>
+        <v>3077</v>
       </c>
       <c r="K236" s="3">
         <f t="shared" si="16"/>
-        <v>5.7323619631901845</v>
+        <v>5.1348716282092948</v>
       </c>
       <c r="L236" s="2">
-        <v>1581</v>
+        <v>951</v>
       </c>
     </row>
     <row r="237" spans="1:12" x14ac:dyDescent="0.25">
@@ -15406,26 +15407,26 @@
         <v>51204</v>
       </c>
       <c r="F238" s="2">
-        <v>1581</v>
+        <v>630</v>
       </c>
       <c r="G238" s="2">
-        <v>1375</v>
+        <v>526</v>
       </c>
       <c r="H238" s="2">
-        <v>1961</v>
+        <v>842</v>
       </c>
       <c r="I238" s="2">
-        <v>299</v>
+        <v>141</v>
       </c>
       <c r="J238" s="2">
-        <v>5216</v>
+        <v>2139</v>
       </c>
       <c r="K238" s="3">
         <f t="shared" ref="K238" si="17">(I238/J238)*100</f>
-        <v>5.7323619631901845</v>
+        <v>6.5918653576437585</v>
       </c>
       <c r="L238" s="2">
-        <v>1581</v>
+        <v>630</v>
       </c>
     </row>
     <row r="239" spans="1:12" x14ac:dyDescent="0.25">
@@ -16108,26 +16109,26 @@
         <v>70101</v>
       </c>
       <c r="F256" s="2">
-        <v>523</v>
+        <v>451</v>
       </c>
       <c r="G256" s="2">
-        <v>5319</v>
+        <v>5058</v>
       </c>
       <c r="H256" s="2">
-        <v>163447</v>
+        <v>161414</v>
       </c>
       <c r="I256" s="2">
-        <v>193588</v>
+        <v>193518</v>
       </c>
       <c r="J256" s="2">
-        <v>362877</v>
+        <v>360441</v>
       </c>
       <c r="K256" s="3">
         <f t="shared" si="16"/>
-        <v>53.348104178550862</v>
+        <v>53.689230692401814</v>
       </c>
       <c r="L256" s="2">
-        <v>523</v>
+        <v>451</v>
       </c>
     </row>
     <row r="257" spans="1:12" x14ac:dyDescent="0.25">
@@ -16147,26 +16148,26 @@
         <v>70102</v>
       </c>
       <c r="F257" s="2">
-        <v>96</v>
+        <v>168</v>
       </c>
       <c r="G257" s="2">
-        <v>697</v>
+        <v>958</v>
       </c>
       <c r="H257" s="2">
-        <v>4864</v>
+        <v>6897</v>
       </c>
       <c r="I257" s="2">
-        <v>4584</v>
+        <v>4654</v>
       </c>
       <c r="J257" s="2">
-        <v>10241</v>
+        <v>12677</v>
       </c>
       <c r="K257" s="3">
         <f t="shared" si="16"/>
-        <v>44.761253783810176</v>
+        <v>36.712155872840583</v>
       </c>
       <c r="L257" s="2">
-        <v>96</v>
+        <v>168</v>
       </c>
     </row>
     <row r="258" spans="1:12" x14ac:dyDescent="0.25">
@@ -17785,26 +17786,26 @@
         <v>71103</v>
       </c>
       <c r="F299" s="2">
-        <v>43</v>
+        <v>523</v>
       </c>
       <c r="G299" s="2">
-        <v>100</v>
+        <v>2212</v>
       </c>
       <c r="H299" s="2">
-        <v>308</v>
+        <v>6716</v>
       </c>
       <c r="I299" s="2">
-        <v>695</v>
+        <v>3316</v>
       </c>
       <c r="J299" s="2">
-        <v>1146</v>
+        <v>12767</v>
       </c>
       <c r="K299" s="3">
         <f t="shared" si="18"/>
-        <v>60.645724258289704</v>
+        <v>25.97321218767134</v>
       </c>
       <c r="L299" s="2">
-        <v>43</v>
+        <v>523</v>
       </c>
     </row>
     <row r="300" spans="1:12" x14ac:dyDescent="0.25">
@@ -17824,26 +17825,26 @@
         <v>71104</v>
       </c>
       <c r="F300" s="2">
-        <v>109</v>
+        <v>43</v>
       </c>
       <c r="G300" s="2">
-        <v>389</v>
+        <v>100</v>
       </c>
       <c r="H300" s="2">
-        <v>1133</v>
+        <v>308</v>
       </c>
       <c r="I300" s="2">
-        <v>54</v>
+        <v>695</v>
       </c>
       <c r="J300" s="2">
-        <v>1685</v>
+        <v>1146</v>
       </c>
       <c r="K300" s="3">
         <f t="shared" si="18"/>
-        <v>3.2047477744807122</v>
+        <v>60.645724258289704</v>
       </c>
       <c r="L300" s="2">
-        <v>109</v>
+        <v>43</v>
       </c>
     </row>
     <row r="301" spans="1:12" x14ac:dyDescent="0.25">
@@ -17863,26 +17864,26 @@
         <v>71105</v>
       </c>
       <c r="F301" s="2">
-        <v>523</v>
+        <v>109</v>
       </c>
       <c r="G301" s="2">
-        <v>2212</v>
+        <v>389</v>
       </c>
       <c r="H301" s="2">
-        <v>6716</v>
+        <v>1133</v>
       </c>
       <c r="I301" s="2">
-        <v>3316</v>
+        <v>54</v>
       </c>
       <c r="J301" s="2">
-        <v>12767</v>
+        <v>1685</v>
       </c>
       <c r="K301" s="3">
         <f t="shared" si="18"/>
-        <v>25.97321218767134</v>
+        <v>3.2047477744807122</v>
       </c>
       <c r="L301" s="2">
-        <v>523</v>
+        <v>109</v>
       </c>
     </row>
     <row r="302" spans="1:12" x14ac:dyDescent="0.25">
@@ -18604,26 +18605,26 @@
         <v>80401</v>
       </c>
       <c r="F320" s="2">
-        <v>218</v>
+        <v>182</v>
       </c>
       <c r="G320" s="2">
-        <v>607</v>
+        <v>504</v>
       </c>
       <c r="H320" s="2">
-        <v>1475</v>
+        <v>1333</v>
       </c>
       <c r="I320" s="2">
-        <v>1412</v>
+        <v>1411</v>
       </c>
       <c r="J320" s="2">
-        <v>3712</v>
+        <v>3430</v>
       </c>
       <c r="K320" s="3">
         <f t="shared" si="18"/>
-        <v>38.038793103448278</v>
+        <v>41.137026239067055</v>
       </c>
       <c r="L320" s="2">
-        <v>218</v>
+        <v>182</v>
       </c>
     </row>
     <row r="321" spans="1:12" x14ac:dyDescent="0.25">
@@ -18682,26 +18683,26 @@
         <v>80501</v>
       </c>
       <c r="F322" s="2">
-        <v>646</v>
+        <v>554</v>
       </c>
       <c r="G322" s="2">
-        <v>1957</v>
+        <v>1824</v>
       </c>
       <c r="H322" s="2">
-        <v>1376</v>
+        <v>1262</v>
       </c>
       <c r="I322" s="2">
-        <v>375</v>
+        <v>365</v>
       </c>
       <c r="J322" s="2">
-        <v>4354</v>
+        <v>4005</v>
       </c>
       <c r="K322" s="3">
         <f t="shared" si="18"/>
-        <v>8.6127698667891597</v>
+        <v>9.1136079900124844</v>
       </c>
       <c r="L322" s="2">
-        <v>646</v>
+        <v>554</v>
       </c>
     </row>
     <row r="323" spans="1:12" x14ac:dyDescent="0.25">
@@ -18931,7 +18932,7 @@
         <v>2232</v>
       </c>
       <c r="K328" s="3">
-        <f t="shared" ref="K328:K347" si="19">(I328/J328)*100</f>
+        <f t="shared" ref="K328:K346" si="19">(I328/J328)*100</f>
         <v>3.4050179211469538</v>
       </c>
       <c r="L328" s="2">
@@ -19033,31 +19034,26 @@
         <v>80901</v>
       </c>
       <c r="F331" s="2">
-        <f>AVERAGE(F322,F320)</f>
-        <v>432</v>
+        <v>128</v>
       </c>
       <c r="G331" s="2">
-        <f>AVERAGE(G322,G320)</f>
-        <v>1282</v>
+        <v>236</v>
       </c>
       <c r="H331" s="2">
-        <f t="shared" ref="H331:J331" si="20">AVERAGE(H322,H320)</f>
-        <v>1425.5</v>
+        <v>256</v>
       </c>
       <c r="I331" s="2">
-        <f t="shared" si="20"/>
-        <v>893.5</v>
+        <v>11</v>
       </c>
       <c r="J331" s="2">
-        <f t="shared" si="20"/>
-        <v>4033</v>
+        <v>631</v>
       </c>
       <c r="K331" s="3">
         <f>(I331/J331)*100</f>
-        <v>22.154723530870321</v>
+        <v>1.7432646592709984</v>
       </c>
       <c r="L331" s="2">
-        <v>864</v>
+        <v>128</v>
       </c>
     </row>
     <row r="332" spans="1:12" x14ac:dyDescent="0.25">
@@ -19657,26 +19653,27 @@
         <v>801</v>
       </c>
       <c r="G347" s="55">
-        <f t="shared" ref="G347:J347" si="21">SUM(G248:G250)</f>
+        <f t="shared" ref="G347:J347" si="20">SUM(G248:G250)</f>
         <v>3083</v>
       </c>
       <c r="H347" s="55">
-        <f t="shared" si="21"/>
+        <f t="shared" si="20"/>
         <v>8836</v>
       </c>
       <c r="I347" s="55">
-        <f t="shared" si="21"/>
+        <f t="shared" si="20"/>
         <v>23702</v>
       </c>
       <c r="J347" s="55">
-        <f t="shared" si="21"/>
+        <f t="shared" si="20"/>
         <v>36422</v>
       </c>
       <c r="K347" s="3">
-        <f t="shared" si="19"/>
+        <f>(I347/J347)*100</f>
         <v>65.076052935039257</v>
       </c>
-      <c r="L347" s="2">
+      <c r="L347" s="55">
+        <f>SUM(L248:L250)</f>
         <v>801</v>
       </c>
       <c r="M347" s="53"/>
@@ -46615,7 +46612,7 @@
         <v>710</v>
       </c>
       <c r="C2" s="3">
-        <v>77.817713181069664</v>
+        <v>77.732347853436082</v>
       </c>
       <c r="D2" s="3">
         <v>83.436902227361642</v>
@@ -46643,7 +46640,7 @@
         <v>754</v>
       </c>
       <c r="C4" s="3">
-        <v>4.1879468845760979</v>
+        <v>3.7768240343347639</v>
       </c>
       <c r="D4" s="3">
         <v>12.849162011173185</v>
@@ -47049,7 +47046,7 @@
         <v>622</v>
       </c>
       <c r="C33" s="3">
-        <v>32.017362546506824</v>
+        <v>32.439228834870079</v>
       </c>
       <c r="D33" s="3">
         <v>56.504599211563736</v>
@@ -47063,7 +47060,7 @@
         <v>624</v>
       </c>
       <c r="C34" s="3">
-        <v>6.7748764996471422</v>
+        <v>6.7263319815410432</v>
       </c>
       <c r="D34" s="3">
         <v>14.057802049456955</v>
@@ -47119,7 +47116,7 @@
         <v>695</v>
       </c>
       <c r="C38" s="3">
-        <v>51.925391095066189</v>
+        <v>22.596299666363361</v>
       </c>
       <c r="D38" s="3">
         <v>49.410870391486128</v>
@@ -47133,7 +47130,7 @@
         <v>694</v>
       </c>
       <c r="C39" s="3">
-        <v>29.478346456692911</v>
+        <v>34.737951013958387</v>
       </c>
       <c r="D39" s="3">
         <v>50.707785642062689</v>
@@ -47147,7 +47144,7 @@
         <v>687</v>
       </c>
       <c r="C40" s="3">
-        <v>22.596299666363361</v>
+        <v>51.925391095066189</v>
       </c>
       <c r="D40" s="3">
         <v>56.954677383344496</v>
@@ -47161,7 +47158,7 @@
         <v>620</v>
       </c>
       <c r="C41" s="3">
-        <v>34.737951013958387</v>
+        <v>29.478346456692911</v>
       </c>
       <c r="D41" s="3">
         <v>70.665603826225592</v>
@@ -47861,7 +47858,7 @@
         <v>564</v>
       </c>
       <c r="C91" s="3">
-        <v>18.625130196004168</v>
+        <v>17.894074273896234</v>
       </c>
       <c r="D91" s="3">
         <v>33.738757630830882</v>
@@ -47903,7 +47900,7 @@
         <v>688</v>
       </c>
       <c r="C94" s="3">
-        <v>12.620357634112791</v>
+        <v>14.650766609880749</v>
       </c>
       <c r="D94" s="3">
         <v>35.225846925972398</v>
@@ -48743,7 +48740,7 @@
         <v>417</v>
       </c>
       <c r="C154" s="3">
-        <v>15.371002401719124</v>
+        <v>20.135135135135133</v>
       </c>
       <c r="D154" s="3">
         <v>41.997383340601829</v>
@@ -48785,7 +48782,7 @@
         <v>794</v>
       </c>
       <c r="C157" s="3">
-        <v>15.371002401719124</v>
+        <v>1.2054244098442994</v>
       </c>
       <c r="D157" s="3">
         <v>9.4553706505295008</v>
@@ -48967,7 +48964,7 @@
         <v>784</v>
       </c>
       <c r="C170" s="3">
-        <v>23.839073327127934</v>
+        <v>23.569330497315914</v>
       </c>
       <c r="D170" s="3">
         <v>37.059735656796875</v>
@@ -49331,7 +49328,7 @@
         <v>464</v>
       </c>
       <c r="C196" s="3">
-        <v>18.974700399467377</v>
+        <v>19.363086936308694</v>
       </c>
       <c r="D196" s="3">
         <v>32.938133218366026</v>
@@ -49555,7 +49552,7 @@
         <v>531</v>
       </c>
       <c r="C212" s="3">
-        <v>14.018779342723004</v>
+        <v>15.748950069995335</v>
       </c>
       <c r="D212" s="3">
         <v>26.997075573341544</v>
@@ -49569,7 +49566,7 @@
         <v>786</v>
       </c>
       <c r="C213" s="3">
-        <v>15.935405240706885</v>
+        <v>15.646970830216903</v>
       </c>
       <c r="D213" s="3">
         <v>21.133720930232556</v>
@@ -49863,7 +49860,7 @@
         <v>452</v>
       </c>
       <c r="C234" s="3">
-        <v>5.7323619631901845</v>
+        <v>5.1348716282092948</v>
       </c>
       <c r="D234" s="3">
         <v>23.33433825746156</v>
@@ -49891,7 +49888,7 @@
         <v>796</v>
       </c>
       <c r="C236" s="3">
-        <v>5.7323619631901845</v>
+        <v>6.5918653576437585</v>
       </c>
       <c r="D236" s="3">
         <v>28.346758726505563</v>
@@ -50143,7 +50140,7 @@
         <v>509</v>
       </c>
       <c r="C254" s="3">
-        <v>53.348104178550862</v>
+        <v>53.689230692401814</v>
       </c>
       <c r="D254" s="3">
         <v>70.494397097701025</v>
@@ -50157,7 +50154,7 @@
         <v>715</v>
       </c>
       <c r="C255" s="3">
-        <v>44.761253783810176</v>
+        <v>36.712155872840583</v>
       </c>
       <c r="D255" s="3">
         <v>27.779973412855242</v>
@@ -50745,7 +50742,7 @@
         <v>529</v>
       </c>
       <c r="C297" s="3">
-        <v>60.645724258289704</v>
+        <v>25.97321218767134</v>
       </c>
       <c r="D297" s="3">
         <v>17.550349362926429</v>
@@ -50759,7 +50756,7 @@
         <v>772</v>
       </c>
       <c r="C298" s="3">
-        <v>3.2047477744807122</v>
+        <v>60.645724258289704</v>
       </c>
       <c r="D298" s="3">
         <v>39.001937984496124</v>
@@ -50773,7 +50770,7 @@
         <v>751</v>
       </c>
       <c r="C299" s="3">
-        <v>25.97321218767134</v>
+        <v>3.2047477744807122</v>
       </c>
       <c r="D299" s="3">
         <v>84.813559322033896</v>
@@ -51039,7 +51036,7 @@
         <v>670</v>
       </c>
       <c r="C318" s="3">
-        <v>38.038793103448278</v>
+        <v>41.137026239067055</v>
       </c>
       <c r="D318" s="3">
         <v>56.088474970896399</v>
@@ -51067,7 +51064,7 @@
         <v>510</v>
       </c>
       <c r="C320" s="3">
-        <v>8.6127698667891597</v>
+        <v>9.1136079900124844</v>
       </c>
       <c r="D320" s="3">
         <v>29.104062326099054</v>
@@ -51193,7 +51190,7 @@
         <v>793</v>
       </c>
       <c r="C329" s="3">
-        <v>22.154723530870321</v>
+        <v>1.7432646592709984</v>
       </c>
       <c r="D329" s="3">
         <v>40.997830802603033</v>
@@ -51419,7 +51416,7 @@
   <sheetPr>
     <tabColor rgb="FFC00000"/>
   </sheetPr>
-  <dimension ref="A1:D345"/>
+  <dimension ref="A1:D344"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="14.28515625" customWidth="1"/>
@@ -51449,7 +51446,7 @@
         <v>710</v>
       </c>
       <c r="C2" s="2">
-        <v>3414</v>
+        <v>3453</v>
       </c>
       <c r="D2" s="2">
         <v>1401</v>
@@ -51477,7 +51474,7 @@
         <v>754</v>
       </c>
       <c r="C4" s="2">
-        <v>2634</v>
+        <v>2544</v>
       </c>
       <c r="D4" s="2">
         <v>1195</v>
@@ -51883,7 +51880,7 @@
         <v>622</v>
       </c>
       <c r="C33" s="2">
-        <v>508</v>
+        <v>504</v>
       </c>
       <c r="D33" s="2">
         <v>192</v>
@@ -51897,7 +51894,7 @@
         <v>624</v>
       </c>
       <c r="C34" s="2">
-        <v>1231</v>
+        <v>1235</v>
       </c>
       <c r="D34" s="2">
         <v>1130</v>
@@ -51953,7 +51950,7 @@
         <v>695</v>
       </c>
       <c r="C38" s="2">
-        <v>83</v>
+        <v>547</v>
       </c>
       <c r="D38" s="2">
         <v>171</v>
@@ -51967,7 +51964,7 @@
         <v>694</v>
       </c>
       <c r="C39" s="2">
-        <v>193</v>
+        <v>485</v>
       </c>
       <c r="D39" s="2">
         <v>257</v>
@@ -51981,7 +51978,7 @@
         <v>687</v>
       </c>
       <c r="C40" s="2">
-        <v>547</v>
+        <v>83</v>
       </c>
       <c r="D40" s="2">
         <v>214</v>
@@ -51995,7 +51992,7 @@
         <v>620</v>
       </c>
       <c r="C41" s="2">
-        <v>485</v>
+        <v>193</v>
       </c>
       <c r="D41" s="2">
         <v>113</v>
@@ -52695,7 +52692,7 @@
         <v>564</v>
       </c>
       <c r="C91" s="2">
-        <v>2291</v>
+        <v>2422</v>
       </c>
       <c r="D91" s="2">
         <v>1891</v>
@@ -52737,7 +52734,7 @@
         <v>688</v>
       </c>
       <c r="C94" s="2">
-        <v>341</v>
+        <v>210</v>
       </c>
       <c r="D94" s="2">
         <v>215</v>
@@ -53577,7 +53574,7 @@
         <v>417</v>
       </c>
       <c r="C154" s="2">
-        <v>2582</v>
+        <v>1333</v>
       </c>
       <c r="D154" s="2">
         <v>506</v>
@@ -53619,7 +53616,7 @@
         <v>794</v>
       </c>
       <c r="C157" s="2">
-        <v>2582</v>
+        <v>1249</v>
       </c>
       <c r="D157" s="2">
         <v>968</v>
@@ -53801,7 +53798,7 @@
         <v>784</v>
       </c>
       <c r="C170" s="2">
-        <v>1808</v>
+        <v>1815</v>
       </c>
       <c r="D170" s="2">
         <v>1152</v>
@@ -54165,7 +54162,7 @@
         <v>464</v>
       </c>
       <c r="C196" s="2">
-        <v>1140</v>
+        <v>1133</v>
       </c>
       <c r="D196" s="2">
         <v>574</v>
@@ -54389,7 +54386,7 @@
         <v>531</v>
       </c>
       <c r="C212" s="2">
-        <v>2161</v>
+        <v>919</v>
       </c>
       <c r="D212" s="2">
         <v>930</v>
@@ -54403,7 +54400,7 @@
         <v>786</v>
       </c>
       <c r="C213" s="2">
-        <v>1613</v>
+        <v>1664</v>
       </c>
       <c r="D213" s="2">
         <v>1037</v>
@@ -54445,7 +54442,7 @@
         <v>795</v>
       </c>
       <c r="C216" s="2">
-        <v>2161</v>
+        <v>1242</v>
       </c>
       <c r="D216" s="2">
         <v>1058</v>
@@ -54697,7 +54694,7 @@
         <v>452</v>
       </c>
       <c r="C234" s="2">
-        <v>1581</v>
+        <v>951</v>
       </c>
       <c r="D234" s="2">
         <v>441</v>
@@ -54725,7 +54722,7 @@
         <v>796</v>
       </c>
       <c r="C236" s="2">
-        <v>1581</v>
+        <v>630</v>
       </c>
       <c r="D236" s="2">
         <v>412</v>
@@ -54977,7 +54974,7 @@
         <v>509</v>
       </c>
       <c r="C254" s="2">
-        <v>523</v>
+        <v>451</v>
       </c>
       <c r="D254" s="2">
         <v>388</v>
@@ -54991,7 +54988,7 @@
         <v>715</v>
       </c>
       <c r="C255" s="2">
-        <v>96</v>
+        <v>168</v>
       </c>
       <c r="D255" s="2">
         <v>169</v>
@@ -55579,7 +55576,7 @@
         <v>529</v>
       </c>
       <c r="C297" s="2">
-        <v>43</v>
+        <v>523</v>
       </c>
       <c r="D297" s="2">
         <v>32</v>
@@ -55593,7 +55590,7 @@
         <v>772</v>
       </c>
       <c r="C298" s="2">
-        <v>109</v>
+        <v>43</v>
       </c>
       <c r="D298" s="2">
         <v>231</v>
@@ -55607,7 +55604,7 @@
         <v>751</v>
       </c>
       <c r="C299" s="2">
-        <v>523</v>
+        <v>109</v>
       </c>
       <c r="D299" s="2">
         <v>4</v>
@@ -55873,7 +55870,7 @@
         <v>670</v>
       </c>
       <c r="C318" s="2">
-        <v>218</v>
+        <v>182</v>
       </c>
       <c r="D318" s="2">
         <v>220</v>
@@ -55901,7 +55898,7 @@
         <v>510</v>
       </c>
       <c r="C320" s="2">
-        <v>646</v>
+        <v>554</v>
       </c>
       <c r="D320" s="2">
         <v>308</v>
@@ -56027,7 +56024,7 @@
         <v>793</v>
       </c>
       <c r="C329" s="2">
-        <v>864</v>
+        <v>128</v>
       </c>
       <c r="D329" s="2">
         <v>193</v>
@@ -56241,11 +56238,6 @@
       </c>
       <c r="D344" s="2">
         <v>24</v>
-      </c>
-    </row>
-    <row r="345" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D345">
-        <v>373</v>
       </c>
     </row>
   </sheetData>
@@ -56301,7 +56293,7 @@
         <v>20</v>
       </c>
       <c r="C4" s="23">
-        <v>50.12383323790629</v>
+        <v>50.164244641227071</v>
       </c>
       <c r="D4" s="3">
         <v>64.304829457909165</v>
@@ -56329,7 +56321,7 @@
         <v>3</v>
       </c>
       <c r="C6" s="23">
-        <v>41.788190704245224</v>
+        <v>42.192726399900891</v>
       </c>
       <c r="D6" s="3">
         <v>51.03693871988434</v>
@@ -56357,7 +56349,7 @@
         <v>2</v>
       </c>
       <c r="C8" s="23">
-        <v>34.839002197274141</v>
+        <v>36.363298693366133</v>
       </c>
       <c r="D8" s="3">
         <v>46.350721822581441</v>
@@ -56399,7 +56391,7 @@
         <v>27</v>
       </c>
       <c r="C11" s="23">
-        <v>20.876652673702381</v>
+        <v>20.766854830120355</v>
       </c>
       <c r="D11" s="3">
         <v>28.566015094577953</v>
@@ -56441,7 +56433,7 @@
         <v>1195</v>
       </c>
       <c r="C14" s="23">
-        <v>45.510742023926021</v>
+        <v>45.856571119215459</v>
       </c>
       <c r="D14" s="3">
         <v>57.25012287127754</v>
@@ -56494,7 +56486,7 @@
         <v>20</v>
       </c>
       <c r="C2" s="43">
-        <v>26012</v>
+        <v>25961</v>
       </c>
       <c r="D2" s="21">
         <v>11084</v>
@@ -56522,7 +56514,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="43">
-        <v>59642</v>
+        <v>57060</v>
       </c>
       <c r="D4" s="21">
         <v>40277</v>
@@ -56550,7 +56542,7 @@
         <v>2</v>
       </c>
       <c r="C6" s="43">
-        <v>39275</v>
+        <v>35584</v>
       </c>
       <c r="D6" s="21">
         <v>24693</v>
@@ -56592,7 +56584,7 @@
         <v>27</v>
       </c>
       <c r="C9" s="43">
-        <v>8500</v>
+        <v>7636</v>
       </c>
       <c r="D9" s="21">
         <v>6135</v>
@@ -56634,7 +56626,7 @@
         <v>1195</v>
       </c>
       <c r="C12" s="21">
-        <v>258919</v>
+        <v>251731</v>
       </c>
       <c r="D12" s="21">
         <v>152254</v>

</xml_diff>